<commit_message>
Fix enrich N-row skip, PDF 1x1 fit, unprotected Excel; add usage guide.
Import enrich only fills Y rows and never mutates source; PDF uses PrintCommunication fit; run.bat keeps errors visible; usage guide for operators.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/revize_teklif_sablonu.xlsx
+++ b/assets/templates/revize_teklif_sablonu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus.DESKTOP-9F6EQVL\Desktop\KLDHDH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus.DESKTOP-9F6EQVL\Desktop\teklif-hazirlama\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D991AE0-979C-4D61-A357-05C916B81F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47309017-DD14-479F-A549-1390375F6845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revize Teklif" sheetId="3" r:id="rId1"/>
@@ -107,9 +107,6 @@
     <t>Ara Toplam</t>
   </si>
   <si>
-    <t>Genel hüküm ve şartlar www.antsiselektronik.com.tr/genelhukum-ve-sartlar adresinden indirilebilir.</t>
-  </si>
-  <si>
     <t>Ürünlerin faturası, ürünlerin sevkiyatına mütakip kesilecektir.</t>
   </si>
   <si>
@@ -209,6 +206,9 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>Genel hüküm ve şartlar https://antsiselektronik.com.tr/wp-content/uploads/2024/12/General-Commercial-Terms-and-Conditions.pdf adresinden indirilebilir.</t>
   </si>
 </sst>
 </file>
@@ -613,69 +613,69 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1208,32 +1208,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="6" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55"/>
-      <c r="B1" s="57"/>
-      <c r="C1" s="55" t="s">
+      <c r="A1" s="69"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="69" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="48" t="s">
         <v>38</v>
-      </c>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="48" t="s">
-        <v>39</v>
       </c>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58"/>
-      <c r="B2" s="60"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="60"/>
+      <c r="A2" s="71"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="72"/>
       <c r="G2" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2" s="49">
         <v>45420</v>
@@ -1242,30 +1242,30 @@
       <c r="J2"/>
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="58"/>
-      <c r="B3" s="60"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="60"/>
+      <c r="A3" s="71"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="72"/>
       <c r="G3" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H3" s="50" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I3"/>
       <c r="J3"/>
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58"/>
-      <c r="B4" s="60"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="60"/>
+      <c r="A4" s="71"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="72"/>
       <c r="G4" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H4" s="49">
         <v>45950</v>
@@ -1275,26 +1275,26 @@
       <c r="L4" s="9"/>
     </row>
     <row r="5" spans="1:12" s="6" customFormat="1" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
-      <c r="B5" s="60"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="60"/>
+      <c r="A5" s="71"/>
+      <c r="B5" s="72"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="72"/>
       <c r="G5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="50" t="s">
         <v>36</v>
-      </c>
-      <c r="H5" s="50" t="s">
-        <v>37</v>
       </c>
       <c r="I5"/>
       <c r="J5"/>
       <c r="L5" s="9"/>
     </row>
     <row r="6" spans="1:12" ht="35.4" x14ac:dyDescent="0.6">
-      <c r="A6" s="67"/>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
+      <c r="A6" s="75"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="76"/>
       <c r="D6" s="11"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
@@ -1305,11 +1305,11 @@
       <c r="I6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
+      <c r="B7" s="60"/>
+      <c r="C7" s="60"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
@@ -1324,7 +1324,7 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H8" s="20"/>
     </row>
@@ -1338,7 +1338,7 @@
       <c r="E9" s="6"/>
       <c r="F9" s="21"/>
       <c r="G9" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H9" s="22"/>
     </row>
@@ -1350,10 +1350,10 @@
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
-      <c r="F10" s="76" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="76"/>
+      <c r="F10" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="78"/>
       <c r="H10" s="22"/>
       <c r="I10" s="3"/>
     </row>
@@ -1366,18 +1366,18 @@
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="G11" s="24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="71" t="s">
+      <c r="A12" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="70"/>
-      <c r="C12" s="73"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="79"/>
       <c r="D12" s="23"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="14" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1406,8 +1406,8 @@
       <c r="H14" s="17"/>
     </row>
     <row r="15" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A15" s="71"/>
-      <c r="B15" s="70"/>
+      <c r="A15" s="59"/>
+      <c r="B15" s="60"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -1417,7 +1417,7 @@
     </row>
     <row r="16" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="17" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1441,7 +1441,7 @@
     </row>
     <row r="18" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1452,10 +1452,10 @@
       <c r="H18" s="17"/>
     </row>
     <row r="19" spans="1:8" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="72" t="s">
-        <v>51</v>
-      </c>
-      <c r="B19" s="70"/>
+      <c r="A19" s="61" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="60"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -1487,41 +1487,41 @@
       <c r="A22" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="61" t="s">
+      <c r="B22" s="55" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="62"/>
-      <c r="D22" s="63"/>
+      <c r="D22" s="56"/>
       <c r="E22" s="29" t="s">
         <v>10</v>
       </c>
       <c r="F22" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="77" t="s">
+      <c r="G22" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="H22" s="77"/>
+      <c r="H22" s="63"/>
     </row>
     <row r="23" spans="1:8" s="4" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="64" t="s">
         <v>52</v>
-      </c>
-      <c r="B23" s="64" t="s">
-        <v>53</v>
       </c>
       <c r="C23" s="65"/>
       <c r="D23" s="66"/>
       <c r="E23" s="31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F23" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="G23" s="74" t="s">
-        <v>28</v>
-      </c>
-      <c r="H23" s="75"/>
+      <c r="G23" s="67" t="s">
+        <v>27</v>
+      </c>
+      <c r="H23" s="68"/>
     </row>
     <row r="24" spans="1:8" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A24" s="46"/>
@@ -1548,12 +1548,12 @@
         <v>6</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="61" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D26" s="63"/>
+      <c r="D26" s="56"/>
       <c r="E26" s="29" t="s">
         <v>21</v>
       </c>
@@ -1561,17 +1561,17 @@
         <v>20</v>
       </c>
       <c r="G26" s="33" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H26" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="4" customFormat="1" ht="31.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="34"/>
       <c r="B27" s="34"/>
-      <c r="C27" s="78"/>
-      <c r="D27" s="79"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="58"/>
       <c r="E27" s="35"/>
       <c r="F27" s="52" t="e">
         <f>1-(G27/E27)</f>
@@ -1586,8 +1586,8 @@
     <row r="28" spans="1:8" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="34"/>
       <c r="B28" s="34"/>
-      <c r="C28" s="78"/>
-      <c r="D28" s="79"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="58"/>
       <c r="E28" s="35"/>
       <c r="F28" s="52" t="e">
         <f>1-(G28/E28)</f>
@@ -1622,7 +1622,7 @@
       <c r="E30" s="53"/>
       <c r="F30" s="38"/>
       <c r="G30" s="39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H30" s="35">
         <f>H29*0.2</f>
@@ -1680,7 +1680,7 @@
     </row>
     <row r="35" spans="1:9" s="4" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="54" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B35" s="38"/>
       <c r="C35" s="38"/>
@@ -1692,7 +1692,7 @@
     </row>
     <row r="36" spans="1:9" s="4" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -1705,7 +1705,7 @@
     </row>
     <row r="37" spans="1:9" s="4" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -1718,7 +1718,7 @@
     </row>
     <row r="38" spans="1:9" s="4" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B38" s="38"/>
       <c r="C38" s="38"/>
@@ -1730,7 +1730,7 @@
     </row>
     <row r="39" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="40" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -1764,12 +1764,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="B22:D22"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="G23:H23"/>
@@ -1779,6 +1773,12 @@
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="B22:D22"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.51181102362204722" bottom="0.51181102362204722" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>